<commit_message>
Update customer sample excel file
</commit_message>
<xml_diff>
--- a/customers_sample.xlsx
+++ b/customers_sample.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Learning2025\WebAppDev\AutomateBilingSMS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Learning2025\WebAppDev\AutomateBilingSMS_with_RMS\AutomateBilingSMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Phone Number</t>
   </si>
@@ -42,13 +42,7 @@
     <t>Customer Name</t>
   </si>
   <si>
-    <t>HSE A1</t>
-  </si>
-  <si>
     <t>HSE A2</t>
-  </si>
-  <si>
-    <t>HSE A3</t>
   </si>
 </sst>
 </file>
@@ -394,11 +388,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
     <col min="2" max="2" width="38.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -429,7 +424,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="1">
-        <v>254708538496</v>
+        <v>254784882772</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -444,52 +439,6 @@
         <v>65</v>
       </c>
       <c r="G2">
-        <v>2925</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1">
-        <v>254709538496</v>
-      </c>
-      <c r="C3">
-        <v>100</v>
-      </c>
-      <c r="D3">
-        <v>145</v>
-      </c>
-      <c r="E3">
-        <v>45</v>
-      </c>
-      <c r="F3">
-        <v>65</v>
-      </c>
-      <c r="G3">
-        <v>2925</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1">
-        <v>254733492031</v>
-      </c>
-      <c r="C4">
-        <v>100</v>
-      </c>
-      <c r="D4">
-        <v>145</v>
-      </c>
-      <c r="E4">
-        <v>45</v>
-      </c>
-      <c r="F4">
-        <v>65</v>
-      </c>
-      <c r="G4">
         <v>2925</v>
       </c>
     </row>

</xml_diff>